<commit_message>
Refresh onboarding and retire welcome audio
</commit_message>
<xml_diff>
--- a/output/phrase_review/phrase_catalog.xlsx
+++ b/output/phrase_review/phrase_catalog.xlsx
@@ -128,7 +128,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U247"/>
+  <dimension ref="A1:U231"/>
   <sheetFormatPr defaultRowHeight="20"/>
   <cols>
     <col min="1" max="1" width="8.0" customWidth="1"/>
@@ -263,7 +263,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2">
-        <v>165</v>
+        <v>149</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -292,12 +292,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ease off and regain control.</t>
+          <t xml:space="preserve">Ease back slightly.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Litt ned. Finn kontroll.</t>
+          <t xml:space="preserve">Ro ned litt.</t>
         </is>
       </c>
       <c r="I2" s="3">
@@ -352,7 +352,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2">
-        <v>164</v>
+        <v>148</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
@@ -441,7 +441,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2">
-        <v>169</v>
+        <v>153</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -470,12 +470,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Build effort slightly now.</t>
+          <t xml:space="preserve">Pick it up.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Litt opp i innsats nå.</t>
+          <t xml:space="preserve">Øk litt nå.</t>
         </is>
       </c>
       <c r="I4" s="3">
@@ -530,7 +530,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2">
-        <v>168</v>
+        <v>152</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
@@ -619,7 +619,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2">
-        <v>173</v>
+        <v>157</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
@@ -648,12 +648,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nice. Hold this zone.</t>
+          <t xml:space="preserve">Stay right here.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bra. Hold deg her.</t>
+          <t xml:space="preserve">Bli her.</t>
         </is>
       </c>
       <c r="I6" s="3">
@@ -708,7 +708,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2">
-        <v>172</v>
+        <v>156</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
@@ -742,7 +742,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bra. Hold deg her.</t>
+          <t xml:space="preserve">Bli her.</t>
         </is>
       </c>
       <c r="I7" s="3">
@@ -797,7 +797,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2">
-        <v>192</v>
+        <v>176</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
@@ -826,12 +826,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hold steady rhythm.</t>
+          <t xml:space="preserve">Find your pace.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hold jevn rytme.</t>
+          <t xml:space="preserve">Finn rytmen.</t>
         </is>
       </c>
       <c r="I8" s="3">
@@ -886,7 +886,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2">
-        <v>191</v>
+        <v>175</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
@@ -915,12 +915,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stay easy between reps.</t>
+          <t xml:space="preserve">Relax your shoulders.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rolig mellom dragene.</t>
+          <t xml:space="preserve">Senk skuldrene.</t>
         </is>
       </c>
       <c r="I9" s="3">
@@ -975,7 +975,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2">
-        <v>190</v>
+        <v>174</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -1004,12 +1004,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stay controlled. Rep by rep.</t>
+          <t xml:space="preserve">Hold the rhythm.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hold kontroll. Ett drag av gangen.</t>
+          <t xml:space="preserve">Hold rytmen.</t>
         </is>
       </c>
       <c r="I10" s="3">
@@ -1064,7 +1064,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2">
-        <v>189</v>
+        <v>173</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -1093,12 +1093,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drive the pace now.</t>
+          <t xml:space="preserve">Final push now!</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trykk til nå.</t>
+          <t xml:space="preserve">Trykk til nå!</t>
         </is>
       </c>
       <c r="I11" s="3">
@@ -1153,7 +1153,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2">
-        <v>182</v>
+        <v>166</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -1242,7 +1242,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2">
-        <v>183</v>
+        <v>167</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
@@ -1331,7 +1331,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2">
-        <v>184</v>
+        <v>168</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -1360,12 +1360,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hold this rhythm.</t>
+          <t xml:space="preserve">Stay with the rhythm.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hold denne rytmen.</t>
+          <t xml:space="preserve">Bli i rytmen.</t>
         </is>
       </c>
       <c r="I14" s="3">
@@ -1420,7 +1420,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2">
-        <v>185</v>
+        <v>169</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hold deg rolig og avslappet.</t>
+          <t xml:space="preserve">Rolig og avslappet.</t>
         </is>
       </c>
       <c r="I15" s="3">
@@ -1509,7 +1509,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2">
-        <v>186</v>
+        <v>170</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
@@ -1543,7 +1543,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kontroller innsatsen her.</t>
+          <t xml:space="preserve">Kontroll på innsatsen.</t>
         </is>
       </c>
       <c r="I16" s="3">
@@ -1598,7 +1598,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2">
-        <v>187</v>
+        <v>171</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
@@ -1687,7 +1687,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2">
-        <v>188</v>
+        <v>172</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Let it settle here.</t>
+          <t xml:space="preserve">Hold the phase.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">La det sette seg her.</t>
+          <t xml:space="preserve">Hold det her.</t>
         </is>
       </c>
       <c r="I18" s="3">
@@ -1776,7 +1776,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2">
-        <v>181</v>
+        <v>165</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
@@ -1865,7 +1865,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2">
-        <v>161</v>
+        <v>145</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
@@ -1954,7 +1954,7 @@
     </row>
     <row r="21">
       <c r="A21" s="2">
-        <v>162</v>
+        <v>146</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
@@ -2043,7 +2043,7 @@
     </row>
     <row r="22">
       <c r="A22" s="2">
-        <v>163</v>
+        <v>147</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
@@ -2072,12 +2072,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No heart rate signal. Coaching by timing.</t>
+          <t xml:space="preserve">No heart rate signal. I will continue coaching</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ingen pulssignal. Jeg coacher på timing.</t>
+          <t xml:space="preserve">Ingen pulssignal. Jeg fortsetter å coache</t>
         </is>
       </c>
       <c r="I22" s="3">
@@ -2132,7 +2132,7 @@
     </row>
     <row r="23">
       <c r="A23" s="2">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
@@ -2161,12 +2161,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Main set now. Stay controlled.</t>
+          <t xml:space="preserve">Main set now.</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bra jobba</t>
+          <t xml:space="preserve">Nå er du i hoveddelen.</t>
         </is>
       </c>
       <c r="I23" s="3">
@@ -2221,7 +2221,7 @@
     </row>
     <row r="24">
       <c r="A24" s="2">
-        <v>153</v>
+        <v>137</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
@@ -2250,12 +2250,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No sensors now. Run by feel.</t>
+          <t xml:space="preserve">Coaching by breath.</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ingen sensorer nå. Løp på følelse.</t>
+          <t xml:space="preserve">Coacher med pust.</t>
         </is>
       </c>
       <c r="I24" s="3">
@@ -2310,7 +2310,7 @@
     </row>
     <row r="25">
       <c r="A25" s="2">
-        <v>179</v>
+        <v>163</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
@@ -2339,12 +2339,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paused. Start easy when ready.</t>
+          <t xml:space="preserve">Paused session</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pause. Start rolig når du er klar.</t>
+          <t xml:space="preserve">Pauset økten.</t>
         </is>
       </c>
       <c r="I25" s="3">
@@ -2399,7 +2399,7 @@
     </row>
     <row r="26">
       <c r="A26" s="2">
-        <v>180</v>
+        <v>164</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
@@ -2428,12 +2428,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Good. You're moving again.</t>
+          <t xml:space="preserve">You're moving again.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bra. Du er i gang.</t>
+          <t xml:space="preserve">Du er i gang igjen.</t>
         </is>
       </c>
       <c r="I26" s="3">
@@ -2488,7 +2488,7 @@
     </row>
     <row r="27">
       <c r="A27" s="2">
-        <v>178</v>
+        <v>162</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
@@ -2517,12 +2517,12 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cooldown now. Bring it down.</t>
+          <t xml:space="preserve">Cooldown now.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nedjogg nå. Ro ned.</t>
+          <t xml:space="preserve">Nå roer vi ned.</t>
         </is>
       </c>
       <c r="I27" s="3">
@@ -2577,7 +2577,7 @@
     </row>
     <row r="28">
       <c r="A28" s="2">
-        <v>176</v>
+        <v>160</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
@@ -2606,12 +2606,12 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recovery block. Easy jog.</t>
+          <t xml:space="preserve">Recovery now.</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pauseblokk. Rolig jogg.</t>
+          <t xml:space="preserve">Pause nå.</t>
         </is>
       </c>
       <c r="I28" s="3">
@@ -2666,7 +2666,7 @@
     </row>
     <row r="29">
       <c r="A29" s="2">
-        <v>177</v>
+        <v>161</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
@@ -2695,12 +2695,12 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Warm-up now. Keep it easy.</t>
+          <t xml:space="preserve">Prepare for the session.</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nå er vi i oppvarmingsdelen.</t>
+          <t xml:space="preserve">Forbered deg på økten.</t>
         </is>
       </c>
       <c r="I29" s="3">
@@ -2755,7 +2755,7 @@
     </row>
     <row r="30">
       <c r="A30" s="2">
-        <v>174</v>
+        <v>158</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
@@ -2784,12 +2784,12 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Work block. Controlled hard.</t>
+          <t xml:space="preserve">Work starts now.</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dragstart. Kontroller hardt.</t>
+          <t xml:space="preserve">Nå begynner innsatsen.</t>
         </is>
       </c>
       <c r="I30" s="3">
@@ -2844,7 +2844,7 @@
     </row>
     <row r="31">
       <c r="A31" s="2">
-        <v>175</v>
+        <v>159</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
@@ -2873,12 +2873,12 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">New work block. Controlled hard now.</t>
+          <t xml:space="preserve">Time to work.</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nytt drag. Sterk kontroll nå.</t>
+          <t xml:space="preserve">Nå jobber vi.</t>
         </is>
       </c>
       <c r="I31" s="3">
@@ -2933,7 +2933,7 @@
     </row>
     <row r="32">
       <c r="A32" s="2">
-        <v>152</v>
+        <v>136</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
@@ -2962,12 +2962,12 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Watch lost. I'll coach by timing.</t>
+          <t xml:space="preserve">Watch disconnected</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Klokken falt ut. Jeg coacher på timing.</t>
+          <t xml:space="preserve">Pulsklokken ble frakoblet.</t>
         </is>
       </c>
       <c r="I32" s="3">
@@ -3022,7 +3022,7 @@
     </row>
     <row r="33">
       <c r="A33" s="2">
-        <v>154</v>
+        <v>138</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
@@ -3051,12 +3051,12 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Watch back. Zone coaching is back.</t>
+          <t xml:space="preserve">Watch connected and heart rate is back.</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Klokken er tilbake. Sonecoaching er tilbake.</t>
+          <t xml:space="preserve">Klokken er tilkoblet, og pulsen er tilbake.</t>
         </is>
       </c>
       <c r="I33" s="3">
@@ -3111,7 +3111,7 @@
     </row>
     <row r="34">
       <c r="A34" s="2">
-        <v>156</v>
+        <v>140</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
@@ -3140,12 +3140,12 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">15 seconds left.</t>
+          <t xml:space="preserve">15!</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">15</t>
+          <t xml:space="preserve">15!</t>
         </is>
       </c>
       <c r="I34" s="3">
@@ -3200,7 +3200,7 @@
     </row>
     <row r="35">
       <c r="A35" s="2">
-        <v>155</v>
+        <v>139</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
@@ -3234,7 +3234,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">30 sekunder igjen.</t>
+          <t xml:space="preserve">30 sekunder.</t>
         </is>
       </c>
       <c r="I35" s="3">
@@ -3289,7 +3289,7 @@
     </row>
     <row r="36">
       <c r="A36" s="2">
-        <v>157</v>
+        <v>141</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
@@ -3318,12 +3318,12 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 seconds left.</t>
+          <t xml:space="preserve">5!</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">fem</t>
         </is>
       </c>
       <c r="I36" s="3">
@@ -3378,7 +3378,7 @@
     </row>
     <row r="37">
       <c r="A37" s="2">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
@@ -3407,12 +3407,12 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Next interval now.</t>
+          <t xml:space="preserve">Go!</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kjør på nå</t>
+          <t xml:space="preserve">Kjør på nå.</t>
         </is>
       </c>
       <c r="I37" s="3">
@@ -3467,7 +3467,7 @@
     </row>
     <row r="38">
       <c r="A38" s="2">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
@@ -3556,7 +3556,7 @@
     </row>
     <row r="39">
       <c r="A39" s="2">
-        <v>245</v>
+        <v>229</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
@@ -3585,12 +3585,12 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Keep focused on your breath.</t>
+          <t xml:space="preserve">Stay smooth.</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hold fokuset på pusten.</t>
+          <t xml:space="preserve">Hold det rolig.</t>
         </is>
       </c>
       <c r="I39" s="3">
@@ -3645,7 +3645,7 @@
     </row>
     <row r="40">
       <c r="A40" s="2">
-        <v>246</v>
+        <v>230</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
@@ -3674,12 +3674,12 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nice work.</t>
+          <t xml:space="preserve">Keep it steady.</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Herlig jobba!</t>
+          <t xml:space="preserve">Hold det jevnt.</t>
         </is>
       </c>
       <c r="I40" s="3">
@@ -3734,7 +3734,7 @@
     </row>
     <row r="41">
       <c r="A41" s="2">
-        <v>237</v>
+        <v>221</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
@@ -3763,12 +3763,12 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVERYTHING. NOW.</t>
+          <t xml:space="preserve">Finish strong!</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALT. NÅ.</t>
+          <t xml:space="preserve">Kjør på nå!</t>
         </is>
       </c>
       <c r="I41" s="3">
@@ -3823,7 +3823,7 @@
     </row>
     <row r="42">
       <c r="A42" s="2">
-        <v>238</v>
+        <v>222</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
@@ -3852,12 +3852,12 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">COME ON! All the way!</t>
+          <t xml:space="preserve">All the way in.</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KOM IGJEN! Helt inn nå!</t>
+          <t xml:space="preserve">Helt inn!</t>
         </is>
       </c>
       <c r="I42" s="3">
@@ -3912,7 +3912,7 @@
     </row>
     <row r="43">
       <c r="A43" s="2">
-        <v>204</v>
+        <v>188</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
@@ -3941,12 +3941,12 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Perfect.</t>
+          <t xml:space="preserve">Nice work!</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Herlig!</t>
+          <t xml:space="preserve">Hold det sterkt.</t>
         </is>
       </c>
       <c r="I43" s="3">
@@ -4001,7 +4001,7 @@
     </row>
     <row r="44">
       <c r="A44" s="2">
-        <v>213</v>
+        <v>197</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
@@ -4090,7 +4090,7 @@
     </row>
     <row r="45">
       <c r="A45" s="2">
-        <v>205</v>
+        <v>189</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
@@ -4124,7 +4124,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Perfekt!</t>
+          <t xml:space="preserve">Bra jobba!</t>
         </is>
       </c>
       <c r="I45" s="3">
@@ -4179,7 +4179,7 @@
     </row>
     <row r="46">
       <c r="A46" s="2">
-        <v>206</v>
+        <v>190</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
@@ -4268,7 +4268,7 @@
     </row>
     <row r="47">
       <c r="A47" s="2">
-        <v>207</v>
+        <v>191</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
@@ -4357,7 +4357,7 @@
     </row>
     <row r="48">
       <c r="A48" s="2">
-        <v>208</v>
+        <v>192</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
@@ -4446,7 +4446,7 @@
     </row>
     <row r="49">
       <c r="A49" s="2">
-        <v>209</v>
+        <v>193</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
@@ -4535,7 +4535,7 @@
     </row>
     <row r="50">
       <c r="A50" s="2">
-        <v>210</v>
+        <v>194</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
@@ -4624,7 +4624,7 @@
     </row>
     <row r="51">
       <c r="A51" s="2">
-        <v>211</v>
+        <v>195</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
@@ -4713,7 +4713,7 @@
     </row>
     <row r="52">
       <c r="A52" s="2">
-        <v>212</v>
+        <v>196</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
@@ -4802,7 +4802,7 @@
     </row>
     <row r="53">
       <c r="A53" s="2">
-        <v>243</v>
+        <v>227</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
@@ -4831,12 +4831,12 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Perfect.</t>
+          <t xml:space="preserve">Nice work!</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Perfekt!</t>
+          <t xml:space="preserve">Bra jobba!</t>
         </is>
       </c>
       <c r="I53" s="3">
@@ -4891,7 +4891,7 @@
     </row>
     <row r="54">
       <c r="A54" s="2">
-        <v>244</v>
+        <v>228</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
@@ -4920,7 +4920,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Good work!</t>
+          <t xml:space="preserve">Keep it strong.</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -4980,7 +4980,7 @@
     </row>
     <row r="55">
       <c r="A55" s="2">
-        <v>235</v>
+        <v>219</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
@@ -5009,12 +5009,12 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">You are doing the work!</t>
+          <t xml:space="preserve">Perfect!</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bra. Nå gjør du jobben!</t>
+          <t xml:space="preserve">Hold rytmen.</t>
         </is>
       </c>
       <c r="I55" s="3">
@@ -5069,7 +5069,7 @@
     </row>
     <row r="56">
       <c r="A56" s="2">
-        <v>236</v>
+        <v>220</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
@@ -5098,12 +5098,12 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Keep it smooth and strong.</t>
+          <t xml:space="preserve">Stay with it!</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fokuser på jevnt tempo.</t>
+          <t xml:space="preserve">Stå i det!</t>
         </is>
       </c>
       <c r="I56" s="3">
@@ -5158,7 +5158,7 @@
     </row>
     <row r="57">
       <c r="A57" s="2">
-        <v>239</v>
+        <v>223</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
@@ -5187,12 +5187,12 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Go for it!</t>
+          <t xml:space="preserve">Focus on breath and rhythm.</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kjør på!</t>
+          <t xml:space="preserve">Fokuser på pust og rytme.</t>
         </is>
       </c>
       <c r="I57" s="3">
@@ -5247,7 +5247,7 @@
     </row>
     <row r="58">
       <c r="A58" s="2">
-        <v>240</v>
+        <v>224</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
@@ -5276,12 +5276,12 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ease the pace. Good.</t>
+          <t xml:space="preserve">Settle your pace.</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senk tempoet. Godt.</t>
+          <t xml:space="preserve">Finn ditt tempo.</t>
         </is>
       </c>
       <c r="I58" s="3">
@@ -5336,7 +5336,7 @@
     </row>
     <row r="59">
       <c r="A59" s="2">
-        <v>231</v>
+        <v>215</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
@@ -5365,12 +5365,12 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smooth and steady.</t>
+          <t xml:space="preserve">Control your breath.</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nydelig. Bra tempo.</t>
+          <t xml:space="preserve">Kontroller pusten.</t>
         </is>
       </c>
       <c r="I59" s="3">
@@ -5425,7 +5425,7 @@
     </row>
     <row r="60">
       <c r="A60" s="2">
-        <v>232</v>
+        <v>216</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
@@ -5454,12 +5454,12 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Good. Focus on breathing.</t>
+          <t xml:space="preserve">Good start.</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bra. Fokuser på pusten.</t>
+          <t xml:space="preserve">God start.</t>
         </is>
       </c>
       <c r="I60" s="3">
@@ -5514,7 +5514,7 @@
     </row>
     <row r="61">
       <c r="A61" s="2">
-        <v>241</v>
+        <v>225</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
@@ -5543,12 +5543,12 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Steady pressure. Stay in control.</t>
+          <t xml:space="preserve">Good rhythm.</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hold trykket jevnt. Hold kontrollen.</t>
+          <t xml:space="preserve">Bra rytme.</t>
         </is>
       </c>
       <c r="I61" s="3">
@@ -5603,7 +5603,7 @@
     </row>
     <row r="62">
       <c r="A62" s="2">
-        <v>242</v>
+        <v>226</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
@@ -5632,12 +5632,12 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES!</t>
+          <t xml:space="preserve">Keep it steady.</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">JA!</t>
+          <t xml:space="preserve">Hold det jevnt.</t>
         </is>
       </c>
       <c r="I62" s="3">
@@ -5692,7 +5692,7 @@
     </row>
     <row r="63">
       <c r="A63" s="2">
-        <v>233</v>
+        <v>217</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
@@ -5721,12 +5721,12 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Come on!</t>
+          <t xml:space="preserve">Nice work.</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kom igjen!</t>
+          <t xml:space="preserve">Bra jobba.</t>
         </is>
       </c>
       <c r="I63" s="3">
@@ -5781,7 +5781,7 @@
     </row>
     <row r="64">
       <c r="A64" s="2">
-        <v>234</v>
+        <v>218</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
@@ -5810,12 +5810,12 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lovely!</t>
+          <t xml:space="preserve">Hold the rhythm.</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Herlig!</t>
+          <t xml:space="preserve">Hold det sterkt.</t>
         </is>
       </c>
       <c r="I64" s="3">
@@ -5870,7 +5870,7 @@
     </row>
     <row r="65">
       <c r="A65" s="2">
-        <v>119</v>
+        <v>103</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
@@ -5959,7 +5959,7 @@
     </row>
     <row r="66">
       <c r="A66" s="2">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
@@ -6048,7 +6048,7 @@
     </row>
     <row r="67">
       <c r="A67" s="2">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
@@ -6137,7 +6137,7 @@
     </row>
     <row r="68">
       <c r="A68" s="2">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
@@ -6226,7 +6226,7 @@
     </row>
     <row r="69">
       <c r="A69" s="2">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
@@ -6315,7 +6315,7 @@
     </row>
     <row r="70">
       <c r="A70" s="2">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
@@ -6404,7 +6404,7 @@
     </row>
     <row r="71">
       <c r="A71" s="2">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
@@ -6493,7 +6493,7 @@
     </row>
     <row r="72">
       <c r="A72" s="2">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
@@ -6582,7 +6582,7 @@
     </row>
     <row r="73">
       <c r="A73" s="2">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
@@ -6671,7 +6671,7 @@
     </row>
     <row r="74">
       <c r="A74" s="2">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
@@ -6760,7 +6760,7 @@
     </row>
     <row r="75">
       <c r="A75" s="2">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
@@ -6849,7 +6849,7 @@
     </row>
     <row r="76">
       <c r="A76" s="2">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
@@ -6938,7 +6938,7 @@
     </row>
     <row r="77">
       <c r="A77" s="2">
-        <v>125</v>
+        <v>109</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
@@ -7027,7 +7027,7 @@
     </row>
     <row r="78">
       <c r="A78" s="2">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
@@ -7116,7 +7116,7 @@
     </row>
     <row r="79">
       <c r="A79" s="2">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
@@ -7205,7 +7205,7 @@
     </row>
     <row r="80">
       <c r="A80" s="2">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
@@ -7294,7 +7294,7 @@
     </row>
     <row r="81">
       <c r="A81" s="2">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
@@ -7383,7 +7383,7 @@
     </row>
     <row r="82">
       <c r="A82" s="2">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
@@ -7472,7 +7472,7 @@
     </row>
     <row r="83">
       <c r="A83" s="2">
-        <v>102</v>
+        <v>86</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
@@ -7561,7 +7561,7 @@
     </row>
     <row r="84">
       <c r="A84" s="2">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
@@ -7650,7 +7650,7 @@
     </row>
     <row r="85">
       <c r="A85" s="2">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
@@ -7739,7 +7739,7 @@
     </row>
     <row r="86">
       <c r="A86" s="2">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
@@ -7828,7 +7828,7 @@
     </row>
     <row r="87">
       <c r="A87" s="2">
-        <v>116</v>
+        <v>100</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
@@ -7917,7 +7917,7 @@
     </row>
     <row r="88">
       <c r="A88" s="2">
-        <v>117</v>
+        <v>101</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
@@ -8006,7 +8006,7 @@
     </row>
     <row r="89">
       <c r="A89" s="2">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
@@ -8095,7 +8095,7 @@
     </row>
     <row r="90">
       <c r="A90" s="2">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
@@ -8184,7 +8184,7 @@
     </row>
     <row r="91">
       <c r="A91" s="2">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
@@ -8273,7 +8273,7 @@
     </row>
     <row r="92">
       <c r="A92" s="2">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
@@ -8362,7 +8362,7 @@
     </row>
     <row r="93">
       <c r="A93" s="2">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
@@ -8451,7 +8451,7 @@
     </row>
     <row r="94">
       <c r="A94" s="2">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
@@ -8540,7 +8540,7 @@
     </row>
     <row r="95">
       <c r="A95" s="2">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
@@ -8629,7 +8629,7 @@
     </row>
     <row r="96">
       <c r="A96" s="2">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
@@ -8718,7 +8718,7 @@
     </row>
     <row r="97">
       <c r="A97" s="2">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
@@ -8807,7 +8807,7 @@
     </row>
     <row r="98">
       <c r="A98" s="2">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
@@ -8896,7 +8896,7 @@
     </row>
     <row r="99">
       <c r="A99" s="2">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
@@ -8985,7 +8985,7 @@
     </row>
     <row r="100">
       <c r="A100" s="2">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
@@ -9074,7 +9074,7 @@
     </row>
     <row r="101">
       <c r="A101" s="2">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
@@ -9163,7 +9163,7 @@
     </row>
     <row r="102">
       <c r="A102" s="2">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
@@ -9252,7 +9252,7 @@
     </row>
     <row r="103">
       <c r="A103" s="2">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
@@ -9341,7 +9341,7 @@
     </row>
     <row r="104">
       <c r="A104" s="2">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
@@ -9430,7 +9430,7 @@
     </row>
     <row r="105">
       <c r="A105" s="2">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
@@ -9519,7 +9519,7 @@
     </row>
     <row r="106">
       <c r="A106" s="2">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
@@ -9608,7 +9608,7 @@
     </row>
     <row r="107">
       <c r="A107" s="2">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
@@ -9697,7 +9697,7 @@
     </row>
     <row r="108">
       <c r="A108" s="2">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
@@ -9786,7 +9786,7 @@
     </row>
     <row r="109">
       <c r="A109" s="2">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
@@ -9875,7 +9875,7 @@
     </row>
     <row r="110">
       <c r="A110" s="2">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
@@ -9964,7 +9964,7 @@
     </row>
     <row r="111">
       <c r="A111" s="2">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
@@ -10053,7 +10053,7 @@
     </row>
     <row r="112">
       <c r="A112" s="2">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
@@ -10142,7 +10142,7 @@
     </row>
     <row r="113">
       <c r="A113" s="2">
-        <v>224</v>
+        <v>208</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
@@ -10231,7 +10231,7 @@
     </row>
     <row r="114">
       <c r="A114" s="2">
-        <v>225</v>
+        <v>209</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
@@ -10320,7 +10320,7 @@
     </row>
     <row r="115">
       <c r="A115" s="2">
-        <v>226</v>
+        <v>210</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
@@ -10409,7 +10409,7 @@
     </row>
     <row r="116">
       <c r="A116" s="2">
-        <v>227</v>
+        <v>211</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
@@ -10498,7 +10498,7 @@
     </row>
     <row r="117">
       <c r="A117" s="2">
-        <v>228</v>
+        <v>212</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
@@ -10587,7 +10587,7 @@
     </row>
     <row r="118">
       <c r="A118" s="2">
-        <v>229</v>
+        <v>213</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
@@ -10616,12 +10616,12 @@
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVERYTHING. NOW.</t>
+          <t xml:space="preserve">Finish strong!</t>
         </is>
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ALT. NÅ.</t>
+          <t xml:space="preserve">Kjør på nå!</t>
         </is>
       </c>
       <c r="I118" s="3">
@@ -10676,7 +10676,7 @@
     </row>
     <row r="119">
       <c r="A119" s="2">
-        <v>230</v>
+        <v>214</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
@@ -10705,12 +10705,12 @@
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">COME ON! All the way!</t>
+          <t xml:space="preserve">All the way in.</t>
         </is>
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">KOM IGJEN! Helt inn nå!</t>
+          <t xml:space="preserve">Helt inn!</t>
         </is>
       </c>
       <c r="I119" s="3">
@@ -10765,7 +10765,7 @@
     </row>
     <row r="120">
       <c r="A120" s="2">
-        <v>220</v>
+        <v>204</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
@@ -10794,12 +10794,12 @@
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Come on!</t>
+          <t xml:space="preserve">Nice work.</t>
         </is>
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kom igjen!</t>
+          <t xml:space="preserve">Bra jobba.</t>
         </is>
       </c>
       <c r="I120" s="3">
@@ -10854,7 +10854,7 @@
     </row>
     <row r="121">
       <c r="A121" s="2">
-        <v>221</v>
+        <v>205</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
@@ -10883,12 +10883,12 @@
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES!</t>
+          <t xml:space="preserve">Keep it steady.</t>
         </is>
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">JA!</t>
+          <t xml:space="preserve">Hold det jevnt.</t>
         </is>
       </c>
       <c r="I121" s="3">
@@ -10943,7 +10943,7 @@
     </row>
     <row r="122">
       <c r="A122" s="2">
-        <v>222</v>
+        <v>206</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
@@ -10972,12 +10972,12 @@
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lovely!</t>
+          <t xml:space="preserve">Hold the rhythm.</t>
         </is>
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Herlig!</t>
+          <t xml:space="preserve">Hold rytmen.</t>
         </is>
       </c>
       <c r="I122" s="3">
@@ -11032,7 +11032,7 @@
     </row>
     <row r="123">
       <c r="A123" s="2">
-        <v>223</v>
+        <v>207</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
@@ -11061,12 +11061,12 @@
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Steady pressure. Stay in control.</t>
+          <t xml:space="preserve">Good rhythm.</t>
         </is>
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hold trykket jevnt. Hold kontrollen.</t>
+          <t xml:space="preserve">Bra rytme.</t>
         </is>
       </c>
       <c r="I123" s="3">
@@ -11121,7 +11121,7 @@
     </row>
     <row r="124">
       <c r="A124" s="2">
-        <v>214</v>
+        <v>198</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
@@ -11210,7 +11210,7 @@
     </row>
     <row r="125">
       <c r="A125" s="2">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
@@ -11239,12 +11239,12 @@
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Go for it!</t>
+          <t xml:space="preserve">Focus on breath and rhythm.</t>
         </is>
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kjør på!</t>
+          <t xml:space="preserve">Fokuser på pust og rytme.</t>
         </is>
       </c>
       <c r="I125" s="3">
@@ -11299,7 +11299,7 @@
     </row>
     <row r="126">
       <c r="A126" s="2">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
@@ -11388,7 +11388,7 @@
     </row>
     <row r="127">
       <c r="A127" s="2">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
@@ -11477,7 +11477,7 @@
     </row>
     <row r="128">
       <c r="A128" s="2">
-        <v>218</v>
+        <v>202</v>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
@@ -11506,12 +11506,12 @@
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ease the pace. Good.</t>
+          <t xml:space="preserve">Settle your pace.</t>
         </is>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senk tempoet. Godt.</t>
+          <t xml:space="preserve">Finn ditt tempo.</t>
         </is>
       </c>
       <c r="I128" s="3">
@@ -11566,7 +11566,7 @@
     </row>
     <row r="129">
       <c r="A129" s="2">
-        <v>219</v>
+        <v>203</v>
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
@@ -11655,7 +11655,7 @@
     </row>
     <row r="130">
       <c r="A130" s="2">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
@@ -11744,7 +11744,7 @@
     </row>
     <row r="131">
       <c r="A131" s="2">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
@@ -11833,7 +11833,7 @@
     </row>
     <row r="132">
       <c r="A132" s="2">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
@@ -11922,7 +11922,7 @@
     </row>
     <row r="133">
       <c r="A133" s="2">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
@@ -12011,7 +12011,7 @@
     </row>
     <row r="134">
       <c r="A134" s="2">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
@@ -12100,7 +12100,7 @@
     </row>
     <row r="135">
       <c r="A135" s="2">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
@@ -12189,7 +12189,7 @@
     </row>
     <row r="136">
       <c r="A136" s="2">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
@@ -12278,7 +12278,7 @@
     </row>
     <row r="137">
       <c r="A137" s="2">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
@@ -12367,7 +12367,7 @@
     </row>
     <row r="138">
       <c r="A138" s="2">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
@@ -12456,7 +12456,7 @@
     </row>
     <row r="139">
       <c r="A139" s="2">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
@@ -12545,7 +12545,7 @@
     </row>
     <row r="140">
       <c r="A140" s="2">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
@@ -12634,7 +12634,7 @@
     </row>
     <row r="141">
       <c r="A141" s="2">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
@@ -12723,7 +12723,7 @@
     </row>
     <row r="142">
       <c r="A142" s="2">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
@@ -12812,7 +12812,7 @@
     </row>
     <row r="143">
       <c r="A143" s="2">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
@@ -12901,7 +12901,7 @@
     </row>
     <row r="144">
       <c r="A144" s="2">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
@@ -12990,7 +12990,7 @@
     </row>
     <row r="145">
       <c r="A145" s="2">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
@@ -13079,7 +13079,7 @@
     </row>
     <row r="146">
       <c r="A146" s="2">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
@@ -13168,7 +13168,7 @@
     </row>
     <row r="147">
       <c r="A147" s="2">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
@@ -13257,7 +13257,7 @@
     </row>
     <row r="148">
       <c r="A148" s="2">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
@@ -13346,7 +13346,7 @@
     </row>
     <row r="149">
       <c r="A149" s="2">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
@@ -13435,7 +13435,7 @@
     </row>
     <row r="150">
       <c r="A150" s="2">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
@@ -13524,7 +13524,7 @@
     </row>
     <row r="151">
       <c r="A151" s="2">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
@@ -13613,7 +13613,7 @@
     </row>
     <row r="152">
       <c r="A152" s="2">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
@@ -13702,7 +13702,7 @@
     </row>
     <row r="153">
       <c r="A153" s="2">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
@@ -13791,7 +13791,7 @@
     </row>
     <row r="154">
       <c r="A154" s="2">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
@@ -13880,7 +13880,7 @@
     </row>
     <row r="155">
       <c r="A155" s="2">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
@@ -13969,7 +13969,7 @@
     </row>
     <row r="156">
       <c r="A156" s="2">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
@@ -14058,7 +14058,7 @@
     </row>
     <row r="157">
       <c r="A157" s="2">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
@@ -14147,7 +14147,7 @@
     </row>
     <row r="158">
       <c r="A158" s="2">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
@@ -14236,7 +14236,7 @@
     </row>
     <row r="159">
       <c r="A159" s="2">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
@@ -14325,7 +14325,7 @@
     </row>
     <row r="160">
       <c r="A160" s="2">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
@@ -14414,7 +14414,7 @@
     </row>
     <row r="161">
       <c r="A161" s="2">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
@@ -14503,7 +14503,7 @@
     </row>
     <row r="162">
       <c r="A162" s="2">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
@@ -14592,7 +14592,7 @@
     </row>
     <row r="163">
       <c r="A163" s="2">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
@@ -14681,7 +14681,7 @@
     </row>
     <row r="164">
       <c r="A164" s="2">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
@@ -14770,7 +14770,7 @@
     </row>
     <row r="165">
       <c r="A165" s="2">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
@@ -14859,7 +14859,7 @@
     </row>
     <row r="166">
       <c r="A166" s="2">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
@@ -14948,7 +14948,7 @@
     </row>
     <row r="167">
       <c r="A167" s="2">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
@@ -15037,7 +15037,7 @@
     </row>
     <row r="168">
       <c r="A168" s="2">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
@@ -15126,7 +15126,7 @@
     </row>
     <row r="169">
       <c r="A169" s="2">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
@@ -15215,7 +15215,7 @@
     </row>
     <row r="170">
       <c r="A170" s="2">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
@@ -15304,7 +15304,7 @@
     </row>
     <row r="171">
       <c r="A171" s="2">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
@@ -15393,7 +15393,7 @@
     </row>
     <row r="172">
       <c r="A172" s="2">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
@@ -15482,7 +15482,7 @@
     </row>
     <row r="173">
       <c r="A173" s="2">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="B173" s="2" t="inlineStr">
         <is>
@@ -15571,7 +15571,7 @@
     </row>
     <row r="174">
       <c r="A174" s="2">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
@@ -15660,7 +15660,7 @@
     </row>
     <row r="175">
       <c r="A175" s="2">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="B175" s="2" t="inlineStr">
         <is>
@@ -15749,7 +15749,7 @@
     </row>
     <row r="176">
       <c r="A176" s="2">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="B176" s="2" t="inlineStr">
         <is>
@@ -15838,7 +15838,7 @@
     </row>
     <row r="177">
       <c r="A177" s="2">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="B177" s="2" t="inlineStr">
         <is>
@@ -15927,7 +15927,7 @@
     </row>
     <row r="178">
       <c r="A178" s="2">
-        <v>85</v>
+        <v>69</v>
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
@@ -16016,7 +16016,7 @@
     </row>
     <row r="179">
       <c r="A179" s="2">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
@@ -16105,7 +16105,7 @@
     </row>
     <row r="180">
       <c r="A180" s="2">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
@@ -16194,7 +16194,7 @@
     </row>
     <row r="181">
       <c r="A181" s="2">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="B181" s="2" t="inlineStr">
         <is>
@@ -16283,7 +16283,7 @@
     </row>
     <row r="182">
       <c r="A182" s="2">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
@@ -16372,7 +16372,7 @@
     </row>
     <row r="183">
       <c r="A183" s="2">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="B183" s="2" t="inlineStr">
         <is>
@@ -16461,7 +16461,7 @@
     </row>
     <row r="184">
       <c r="A184" s="2">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="B184" s="2" t="inlineStr">
         <is>
@@ -16550,7 +16550,7 @@
     </row>
     <row r="185">
       <c r="A185" s="2">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="B185" s="2" t="inlineStr">
         <is>
@@ -16639,7 +16639,7 @@
     </row>
     <row r="186">
       <c r="A186" s="2">
-        <v>83</v>
+        <v>67</v>
       </c>
       <c r="B186" s="2" t="inlineStr">
         <is>
@@ -16728,7 +16728,7 @@
     </row>
     <row r="187">
       <c r="A187" s="2">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="B187" s="2" t="inlineStr">
         <is>
@@ -16817,7 +16817,7 @@
     </row>
     <row r="188">
       <c r="A188" s="2">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="B188" s="2" t="inlineStr">
         <is>
@@ -16906,7 +16906,7 @@
     </row>
     <row r="189">
       <c r="A189" s="2">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="B189" s="2" t="inlineStr">
         <is>
@@ -16995,7 +16995,7 @@
     </row>
     <row r="190">
       <c r="A190" s="2">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="B190" s="2" t="inlineStr">
         <is>
@@ -17084,7 +17084,7 @@
     </row>
     <row r="191">
       <c r="A191" s="2">
-        <v>73</v>
+        <v>57</v>
       </c>
       <c r="B191" s="2" t="inlineStr">
         <is>
@@ -17173,7 +17173,7 @@
     </row>
     <row r="192">
       <c r="A192" s="2">
-        <v>129</v>
+        <v>113</v>
       </c>
       <c r="B192" s="2" t="inlineStr">
         <is>
@@ -17262,7 +17262,7 @@
     </row>
     <row r="193">
       <c r="A193" s="2">
-        <v>138</v>
+        <v>122</v>
       </c>
       <c r="B193" s="2" t="inlineStr">
         <is>
@@ -17351,7 +17351,7 @@
     </row>
     <row r="194">
       <c r="A194" s="2">
-        <v>139</v>
+        <v>123</v>
       </c>
       <c r="B194" s="2" t="inlineStr">
         <is>
@@ -17440,7 +17440,7 @@
     </row>
     <row r="195">
       <c r="A195" s="2">
-        <v>140</v>
+        <v>124</v>
       </c>
       <c r="B195" s="2" t="inlineStr">
         <is>
@@ -17529,7 +17529,7 @@
     </row>
     <row r="196">
       <c r="A196" s="2">
-        <v>141</v>
+        <v>125</v>
       </c>
       <c r="B196" s="2" t="inlineStr">
         <is>
@@ -17618,7 +17618,7 @@
     </row>
     <row r="197">
       <c r="A197" s="2">
-        <v>142</v>
+        <v>126</v>
       </c>
       <c r="B197" s="2" t="inlineStr">
         <is>
@@ -17707,7 +17707,7 @@
     </row>
     <row r="198">
       <c r="A198" s="2">
-        <v>143</v>
+        <v>127</v>
       </c>
       <c r="B198" s="2" t="inlineStr">
         <is>
@@ -17796,7 +17796,7 @@
     </row>
     <row r="199">
       <c r="A199" s="2">
-        <v>144</v>
+        <v>128</v>
       </c>
       <c r="B199" s="2" t="inlineStr">
         <is>
@@ -17885,7 +17885,7 @@
     </row>
     <row r="200">
       <c r="A200" s="2">
-        <v>145</v>
+        <v>129</v>
       </c>
       <c r="B200" s="2" t="inlineStr">
         <is>
@@ -17974,7 +17974,7 @@
     </row>
     <row r="201">
       <c r="A201" s="2">
-        <v>146</v>
+        <v>130</v>
       </c>
       <c r="B201" s="2" t="inlineStr">
         <is>
@@ -18063,7 +18063,7 @@
     </row>
     <row r="202">
       <c r="A202" s="2">
-        <v>147</v>
+        <v>131</v>
       </c>
       <c r="B202" s="2" t="inlineStr">
         <is>
@@ -18152,7 +18152,7 @@
     </row>
     <row r="203">
       <c r="A203" s="2">
-        <v>130</v>
+        <v>114</v>
       </c>
       <c r="B203" s="2" t="inlineStr">
         <is>
@@ -18241,7 +18241,7 @@
     </row>
     <row r="204">
       <c r="A204" s="2">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="B204" s="2" t="inlineStr">
         <is>
@@ -18330,7 +18330,7 @@
     </row>
     <row r="205">
       <c r="A205" s="2">
-        <v>132</v>
+        <v>116</v>
       </c>
       <c r="B205" s="2" t="inlineStr">
         <is>
@@ -18419,7 +18419,7 @@
     </row>
     <row r="206">
       <c r="A206" s="2">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="B206" s="2" t="inlineStr">
         <is>
@@ -18508,7 +18508,7 @@
     </row>
     <row r="207">
       <c r="A207" s="2">
-        <v>134</v>
+        <v>118</v>
       </c>
       <c r="B207" s="2" t="inlineStr">
         <is>
@@ -18597,7 +18597,7 @@
     </row>
     <row r="208">
       <c r="A208" s="2">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="B208" s="2" t="inlineStr">
         <is>
@@ -18686,7 +18686,7 @@
     </row>
     <row r="209">
       <c r="A209" s="2">
-        <v>136</v>
+        <v>120</v>
       </c>
       <c r="B209" s="2" t="inlineStr">
         <is>
@@ -18775,7 +18775,7 @@
     </row>
     <row r="210">
       <c r="A210" s="2">
-        <v>137</v>
+        <v>121</v>
       </c>
       <c r="B210" s="2" t="inlineStr">
         <is>
@@ -18864,7 +18864,7 @@
     </row>
     <row r="211">
       <c r="A211" s="2">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="B211" s="2" t="inlineStr">
         <is>
@@ -18953,7 +18953,7 @@
     </row>
     <row r="212">
       <c r="A212" s="2">
-        <v>148</v>
+        <v>132</v>
       </c>
       <c r="B212" s="2" t="inlineStr">
         <is>
@@ -19042,7 +19042,7 @@
     </row>
     <row r="213">
       <c r="A213" s="2">
-        <v>149</v>
+        <v>133</v>
       </c>
       <c r="B213" s="2" t="inlineStr">
         <is>
@@ -19131,7 +19131,7 @@
     </row>
     <row r="214">
       <c r="A214" s="2">
-        <v>150</v>
+        <v>134</v>
       </c>
       <c r="B214" s="2" t="inlineStr">
         <is>
@@ -19220,7 +19220,7 @@
     </row>
     <row r="215">
       <c r="A215" s="2">
-        <v>151</v>
+        <v>135</v>
       </c>
       <c r="B215" s="2" t="inlineStr">
         <is>
@@ -19309,7 +19309,7 @@
     </row>
     <row r="216">
       <c r="A216" s="2">
-        <v>128</v>
+        <v>112</v>
       </c>
       <c r="B216" s="2" t="inlineStr">
         <is>
@@ -19398,21 +19398,21 @@
     </row>
     <row r="217">
       <c r="A217" s="2">
-        <v>1</v>
+        <v>151</v>
       </c>
       <c r="B217" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.1</t>
+          <t xml:space="preserve">zone.above_ease.default.1</t>
         </is>
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard</t>
+          <t xml:space="preserve">zone.above_ease</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.1</t>
+          <t xml:space="preserve">zone.above_ease.default</t>
         </is>
       </c>
       <c r="E217" s="2" t="inlineStr">
@@ -19427,12 +19427,12 @@
       </c>
       <c r="G217" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Let's begin by warming up the body.</t>
+          <t xml:space="preserve">Still high. Ease down 20 seconds.</t>
         </is>
       </c>
       <c r="H217" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Varm opp kroppen</t>
+          <t xml:space="preserve">Fortsatt høy. Ro ned 20 sekunder.</t>
         </is>
       </c>
       <c r="I217" s="3">
@@ -19487,21 +19487,21 @@
     </row>
     <row r="218">
       <c r="A218" s="2">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="B218" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.10</t>
+          <t xml:space="preserve">zone.above_ease.minimal.1</t>
         </is>
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard</t>
+          <t xml:space="preserve">zone.above_ease</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.10</t>
+          <t xml:space="preserve">zone.above_ease.minimal</t>
         </is>
       </c>
       <c r="E218" s="2" t="inlineStr">
@@ -19516,12 +19516,12 @@
       </c>
       <c r="G218" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Let's begin easy. Just getting your body warmed up.</t>
+          <t xml:space="preserve">HR still climbing. Ease down.</t>
         </is>
       </c>
       <c r="H218" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">La oss starte rolig og få kroppen god og varm.</t>
+          <t xml:space="preserve">Pulsen stiger. Rolig ned.</t>
         </is>
       </c>
       <c r="I218" s="3">
@@ -19576,21 +19576,21 @@
     </row>
     <row r="219">
       <c r="A219" s="2">
-        <v>11</v>
+        <v>155</v>
       </c>
       <c r="B219" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.11</t>
+          <t xml:space="preserve">zone.below_push.default.1</t>
         </is>
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard</t>
+          <t xml:space="preserve">zone.below_push</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.11</t>
+          <t xml:space="preserve">zone.below_push.default</t>
         </is>
       </c>
       <c r="E219" s="2" t="inlineStr">
@@ -19605,12 +19605,12 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nice to see you. I'll guide you through the workout.</t>
+          <t xml:space="preserve">You're moving. Pick it up slightly.</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Godt å se deg. Jeg guider deg igjennom dagens økt.</t>
+          <t xml:space="preserve">Du er i gang. Øk litt.</t>
         </is>
       </c>
       <c r="I219" s="3">
@@ -19665,21 +19665,21 @@
     </row>
     <row r="220">
       <c r="A220" s="2">
-        <v>12</v>
+        <v>154</v>
       </c>
       <c r="B220" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.12</t>
+          <t xml:space="preserve">zone.below_push.minimal.1</t>
         </is>
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard</t>
+          <t xml:space="preserve">zone.below_push</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.12</t>
+          <t xml:space="preserve">zone.below_push.minimal</t>
         </is>
       </c>
       <c r="E220" s="2" t="inlineStr">
@@ -19694,12 +19694,12 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Perfect! You're here, that's the hardest part.</t>
+          <t xml:space="preserve">You're moving. Add a little.</t>
         </is>
       </c>
       <c r="H220" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Herlig! Du er her, det er det vanskeligste.</t>
+          <t xml:space="preserve">Du er i gang. Litt opp.</t>
         </is>
       </c>
       <c r="I220" s="3">
@@ -19754,21 +19754,21 @@
     </row>
     <row r="221">
       <c r="A221" s="2">
-        <v>13</v>
+        <v>184</v>
       </c>
       <c r="B221" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.13</t>
+          <t xml:space="preserve">zone.breath.easy_run.1</t>
         </is>
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard</t>
+          <t xml:space="preserve">zone.breath</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.13</t>
+          <t xml:space="preserve">zone.breath.easy_run</t>
         </is>
       </c>
       <c r="E221" s="2" t="inlineStr">
@@ -19783,12 +19783,12 @@
       </c>
       <c r="G221" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Take a moment. Deep breath in, slow breath out.</t>
+          <t xml:space="preserve">Match your breathing to your pace.</t>
         </is>
       </c>
       <c r="H221" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Start denne økten med 5 dype innpust og 5 rolige utpust.</t>
+          <t xml:space="preserve">Tilpass pusten til tempoet.</t>
         </is>
       </c>
       <c r="I221" s="3">
@@ -19843,21 +19843,21 @@
     </row>
     <row r="222">
       <c r="A222" s="2">
-        <v>14</v>
+        <v>185</v>
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.14</t>
+          <t xml:space="preserve">zone.breath.easy_run.2</t>
         </is>
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard</t>
+          <t xml:space="preserve">zone.breath</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.14</t>
+          <t xml:space="preserve">zone.breath.easy_run</t>
         </is>
       </c>
       <c r="E222" s="2" t="inlineStr">
@@ -19872,12 +19872,12 @@
       </c>
       <c r="G222" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Start by finding your breath, and get in the zone.</t>
+          <t xml:space="preserve">Smooth breaths. You're doing well.</t>
         </is>
       </c>
       <c r="H222" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Start med å finne pusten og komme deg inn i sonen.</t>
+          <t xml:space="preserve">Jevn pust. Du gjør det bra.</t>
         </is>
       </c>
       <c r="I222" s="3">
@@ -19932,21 +19932,21 @@
     </row>
     <row r="223">
       <c r="A223" s="2">
-        <v>15</v>
+        <v>187</v>
       </c>
       <c r="B223" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.15</t>
+          <t xml:space="preserve">zone.breath.recovery.1</t>
         </is>
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard</t>
+          <t xml:space="preserve">zone.breath</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.15</t>
+          <t xml:space="preserve">zone.breath.recovery</t>
         </is>
       </c>
       <c r="E223" s="2" t="inlineStr">
@@ -19961,12 +19961,12 @@
       </c>
       <c r="G223" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Let's connect with your breathing first. Everything else follows from there.</t>
+          <t xml:space="preserve">Slow your breathing down.</t>
         </is>
       </c>
       <c r="H223" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Først koble deg på pusten. Alt annet følger derfra.</t>
+          <t xml:space="preserve">Senk pustetakten.</t>
         </is>
       </c>
       <c r="I223" s="3">
@@ -20021,21 +20021,21 @@
     </row>
     <row r="224">
       <c r="A224" s="2">
-        <v>16</v>
+        <v>186</v>
       </c>
       <c r="B224" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.16</t>
+          <t xml:space="preserve">zone.breath.work.1</t>
         </is>
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard</t>
+          <t xml:space="preserve">zone.breath</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.16</t>
+          <t xml:space="preserve">zone.breath.work</t>
         </is>
       </c>
       <c r="E224" s="2" t="inlineStr">
@@ -20050,12 +20050,12 @@
       </c>
       <c r="G224" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Settle your breath, relax your body. We'll build the intensity gradually.</t>
+          <t xml:space="preserve">Breathe through the effort.</t>
         </is>
       </c>
       <c r="H224" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Finn roen i pusten, slapp av kroppen. Vi bygger intensiteten gradvis.</t>
+          <t xml:space="preserve">Herlig</t>
         </is>
       </c>
       <c r="I224" s="3">
@@ -20110,21 +20110,21 @@
     </row>
     <row r="225">
       <c r="A225" s="2">
-        <v>2</v>
+        <v>177</v>
       </c>
       <c r="B225" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.2</t>
+          <t xml:space="preserve">zone.feel.easy_run.1</t>
         </is>
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard</t>
+          <t xml:space="preserve">zone.feel</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.2</t>
+          <t xml:space="preserve">zone.feel.easy_run</t>
         </is>
       </c>
       <c r="E225" s="2" t="inlineStr">
@@ -20139,12 +20139,12 @@
       </c>
       <c r="G225" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ready when you are.</t>
+          <t xml:space="preserve">Steady effort. Stay comfortable.</t>
         </is>
       </c>
       <c r="H225" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Klar når du er. Gjør kroppen klar for dagens trening.</t>
+          <t xml:space="preserve">Jevn innsats. Hold det behagelig.</t>
         </is>
       </c>
       <c r="I225" s="3">
@@ -20199,21 +20199,21 @@
     </row>
     <row r="226">
       <c r="A226" s="2">
-        <v>3</v>
+        <v>178</v>
       </c>
       <c r="B226" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.3</t>
+          <t xml:space="preserve">zone.feel.easy_run.2</t>
         </is>
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard</t>
+          <t xml:space="preserve">zone.feel</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.3</t>
+          <t xml:space="preserve">zone.feel.easy_run</t>
         </is>
       </c>
       <c r="E226" s="2" t="inlineStr">
@@ -20228,12 +20228,12 @@
       </c>
       <c r="G226" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nice to see you. Let's set the tone for a good session.</t>
+          <t xml:space="preserve">Find your rhythm and hold it.</t>
         </is>
       </c>
       <c r="H226" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Herlig å se deg. La oss varme opp ordentlig før økten starter.</t>
+          <t xml:space="preserve">Finn rytmen din og hold den.</t>
         </is>
       </c>
       <c r="I226" s="3">
@@ -20288,21 +20288,21 @@
     </row>
     <row r="227">
       <c r="A227" s="2">
-        <v>4</v>
+        <v>179</v>
       </c>
       <c r="B227" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.4</t>
+          <t xml:space="preserve">zone.feel.easy_run.3</t>
         </is>
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard</t>
+          <t xml:space="preserve">zone.feel</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.4</t>
+          <t xml:space="preserve">zone.feel.easy_run</t>
         </is>
       </c>
       <c r="E227" s="2" t="inlineStr">
@@ -20317,12 +20317,12 @@
       </c>
       <c r="G227" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Let's get moving. Controlled pace to start, then we'll find your rhythm.</t>
+          <t xml:space="preserve">Easy and controlled. You set the pace.</t>
         </is>
       </c>
       <c r="H227" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">La oss komme i gang. Kontrollert tempo til å begynne med.</t>
+          <t xml:space="preserve">Rolig og kontrollert. Du bestemmer tempoet.</t>
         </is>
       </c>
       <c r="I227" s="3">
@@ -20377,21 +20377,21 @@
     </row>
     <row r="228">
       <c r="A228" s="2">
-        <v>5</v>
+        <v>182</v>
       </c>
       <c r="B228" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.5</t>
+          <t xml:space="preserve">zone.feel.recovery.1</t>
         </is>
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard</t>
+          <t xml:space="preserve">zone.feel</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.5</t>
+          <t xml:space="preserve">zone.feel.recovery</t>
         </is>
       </c>
       <c r="E228" s="2" t="inlineStr">
@@ -20406,12 +20406,12 @@
       </c>
       <c r="G228" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Welcome back.</t>
+          <t xml:space="preserve">Ease off. Let your body recover.</t>
         </is>
       </c>
       <c r="H228" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Velkommen tilbake.</t>
+          <t xml:space="preserve">Slipp av. La kroppen hente seg inn.</t>
         </is>
       </c>
       <c r="I228" s="3">
@@ -20466,21 +20466,21 @@
     </row>
     <row r="229">
       <c r="A229" s="2">
-        <v>6</v>
+        <v>183</v>
       </c>
       <c r="B229" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.6</t>
+          <t xml:space="preserve">zone.feel.recovery.2</t>
         </is>
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard</t>
+          <t xml:space="preserve">zone.feel</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.6</t>
+          <t xml:space="preserve">zone.feel.recovery</t>
         </is>
       </c>
       <c r="E229" s="2" t="inlineStr">
@@ -20495,12 +20495,12 @@
       </c>
       <c r="G229" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alright, let's begin.</t>
+          <t xml:space="preserve">Relax and breathe. Recovery counts.</t>
         </is>
       </c>
       <c r="H229" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Velkommen tilbake, la oss begynne.</t>
+          <t xml:space="preserve">Slapp av og pust. Hvile teller.</t>
         </is>
       </c>
       <c r="I229" s="3">
@@ -20555,21 +20555,21 @@
     </row>
     <row r="230">
       <c r="A230" s="2">
-        <v>7</v>
+        <v>180</v>
       </c>
       <c r="B230" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.7</t>
+          <t xml:space="preserve">zone.feel.work.1</t>
         </is>
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard</t>
+          <t xml:space="preserve">zone.feel</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.7</t>
+          <t xml:space="preserve">zone.feel.work</t>
         </is>
       </c>
       <c r="E230" s="2" t="inlineStr">
@@ -20584,12 +20584,12 @@
       </c>
       <c r="G230" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Let's start easy, then slowly increase the intensity.</t>
+          <t xml:space="preserve">Push hard but controlled.</t>
         </is>
       </c>
       <c r="H230" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">La oss starte rolig, vi øker intensiteten når kroppen er varmet opp.</t>
+          <t xml:space="preserve">Hold en jevn rytme</t>
         </is>
       </c>
       <c r="I230" s="3">
@@ -20644,21 +20644,21 @@
     </row>
     <row r="231">
       <c r="A231" s="2">
-        <v>8</v>
+        <v>181</v>
       </c>
       <c r="B231" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.8</t>
+          <t xml:space="preserve">zone.feel.work.2</t>
         </is>
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard</t>
+          <t xml:space="preserve">zone.feel</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">welcome.standard.8</t>
+          <t xml:space="preserve">zone.feel.work</t>
         </is>
       </c>
       <c r="E231" s="2" t="inlineStr">
@@ -20673,12 +20673,12 @@
       </c>
       <c r="G231" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nice to see you. We'll start slowly and keep it simple.</t>
+          <t xml:space="preserve">Strong effort now. Stay focused.</t>
         </is>
       </c>
       <c r="H231" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fint at du er her. Vi starter sakte og holder det enkelt.</t>
+          <t xml:space="preserve">Sterk innsats nå. Hold fokus.</t>
         </is>
       </c>
       <c r="I231" s="3">
@@ -20731,1434 +20731,10 @@
         </is>
       </c>
     </row>
-    <row r="232">
-      <c r="A232" s="2">
-        <v>9</v>
-      </c>
-      <c r="B232" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">welcome.standard.9</t>
-        </is>
-      </c>
-      <c r="C232" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">welcome.standard</t>
-        </is>
-      </c>
-      <c r="D232" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">welcome.standard.9</t>
-        </is>
-      </c>
-      <c r="E232" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">personal_trainer</t>
-        </is>
-      </c>
-      <c r="F232" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">core</t>
-        </is>
-      </c>
-      <c r="G232" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Welcome. Just focus on breathing and moving at your own pace.</t>
-        </is>
-      </c>
-      <c r="H232" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Velkommen. Bare fokuser på pusten og beveg deg i ditt tempo.</t>
-        </is>
-      </c>
-      <c r="I232" s="3">
-        <f>IF(LEN(TRIM(G232))=0,0,LEN(TRIM(G232))-LEN(SUBSTITUTE(TRIM(G232)," ",""))+1)</f>
-      </c>
-      <c r="J232" s="3">
-        <f>IF(LEN(TRIM(H232))=0,0,LEN(TRIM(H232))-LEN(SUBSTITUTE(TRIM(H232)," ",""))+1)</f>
-      </c>
-      <c r="K232" s="3">
-        <f>LEN(G232)</f>
-      </c>
-      <c r="L232" s="3">
-        <f>LEN(H232)</f>
-      </c>
-      <c r="M232" s="3">
-        <f>IF(COUNTIF($G:$G,G232)&gt;1,"DUP","")</f>
-      </c>
-      <c r="N232" s="3">
-        <f>IF(COUNTIF($H:$H,H232)&gt;1,"DUP","")</f>
-      </c>
-      <c r="O232" s="3">
-        <f>IF(LEFT(B232,LEN(C232))=C232,"OK","CHECK")</f>
-      </c>
-      <c r="P232" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Review</t>
-        </is>
-      </c>
-      <c r="Q232" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="R232" s="5">
-        <f>IF(OR(M232="DUP",N232="DUP",O232="CHECK"),"CHECK","")</f>
-      </c>
-      <c r="S232" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="T232" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="U232" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="233">
-      <c r="A233" s="2">
-        <v>167</v>
-      </c>
-      <c r="B233" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.above_ease.default.1</t>
-        </is>
-      </c>
-      <c r="C233" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.above_ease</t>
-        </is>
-      </c>
-      <c r="D233" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.above_ease.default</t>
-        </is>
-      </c>
-      <c r="E233" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">personal_trainer</t>
-        </is>
-      </c>
-      <c r="F233" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">core</t>
-        </is>
-      </c>
-      <c r="G233" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Still high. Ease down 20 seconds.</t>
-        </is>
-      </c>
-      <c r="H233" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fortsatt høy. Ro ned 20 sekunder.</t>
-        </is>
-      </c>
-      <c r="I233" s="3">
-        <f>IF(LEN(TRIM(G233))=0,0,LEN(TRIM(G233))-LEN(SUBSTITUTE(TRIM(G233)," ",""))+1)</f>
-      </c>
-      <c r="J233" s="3">
-        <f>IF(LEN(TRIM(H233))=0,0,LEN(TRIM(H233))-LEN(SUBSTITUTE(TRIM(H233)," ",""))+1)</f>
-      </c>
-      <c r="K233" s="3">
-        <f>LEN(G233)</f>
-      </c>
-      <c r="L233" s="3">
-        <f>LEN(H233)</f>
-      </c>
-      <c r="M233" s="3">
-        <f>IF(COUNTIF($G:$G,G233)&gt;1,"DUP","")</f>
-      </c>
-      <c r="N233" s="3">
-        <f>IF(COUNTIF($H:$H,H233)&gt;1,"DUP","")</f>
-      </c>
-      <c r="O233" s="3">
-        <f>IF(LEFT(B233,LEN(C233))=C233,"OK","CHECK")</f>
-      </c>
-      <c r="P233" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Review</t>
-        </is>
-      </c>
-      <c r="Q233" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="R233" s="5">
-        <f>IF(OR(M233="DUP",N233="DUP",O233="CHECK"),"CHECK","")</f>
-      </c>
-      <c r="S233" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="T233" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="U233" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="234">
-      <c r="A234" s="2">
-        <v>166</v>
-      </c>
-      <c r="B234" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.above_ease.minimal.1</t>
-        </is>
-      </c>
-      <c r="C234" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.above_ease</t>
-        </is>
-      </c>
-      <c r="D234" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.above_ease.minimal</t>
-        </is>
-      </c>
-      <c r="E234" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">personal_trainer</t>
-        </is>
-      </c>
-      <c r="F234" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">core</t>
-        </is>
-      </c>
-      <c r="G234" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HR still climbing. Ease down.</t>
-        </is>
-      </c>
-      <c r="H234" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pulsen stiger. Rolig ned.</t>
-        </is>
-      </c>
-      <c r="I234" s="3">
-        <f>IF(LEN(TRIM(G234))=0,0,LEN(TRIM(G234))-LEN(SUBSTITUTE(TRIM(G234)," ",""))+1)</f>
-      </c>
-      <c r="J234" s="3">
-        <f>IF(LEN(TRIM(H234))=0,0,LEN(TRIM(H234))-LEN(SUBSTITUTE(TRIM(H234)," ",""))+1)</f>
-      </c>
-      <c r="K234" s="3">
-        <f>LEN(G234)</f>
-      </c>
-      <c r="L234" s="3">
-        <f>LEN(H234)</f>
-      </c>
-      <c r="M234" s="3">
-        <f>IF(COUNTIF($G:$G,G234)&gt;1,"DUP","")</f>
-      </c>
-      <c r="N234" s="3">
-        <f>IF(COUNTIF($H:$H,H234)&gt;1,"DUP","")</f>
-      </c>
-      <c r="O234" s="3">
-        <f>IF(LEFT(B234,LEN(C234))=C234,"OK","CHECK")</f>
-      </c>
-      <c r="P234" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Review</t>
-        </is>
-      </c>
-      <c r="Q234" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="R234" s="5">
-        <f>IF(OR(M234="DUP",N234="DUP",O234="CHECK"),"CHECK","")</f>
-      </c>
-      <c r="S234" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="T234" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="U234" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="235">
-      <c r="A235" s="2">
-        <v>171</v>
-      </c>
-      <c r="B235" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.below_push.default.1</t>
-        </is>
-      </c>
-      <c r="C235" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.below_push</t>
-        </is>
-      </c>
-      <c r="D235" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.below_push.default</t>
-        </is>
-      </c>
-      <c r="E235" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">personal_trainer</t>
-        </is>
-      </c>
-      <c r="F235" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">core</t>
-        </is>
-      </c>
-      <c r="G235" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">You're moving. Pick it up slightly.</t>
-        </is>
-      </c>
-      <c r="H235" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du er i gang. Øk litt.</t>
-        </is>
-      </c>
-      <c r="I235" s="3">
-        <f>IF(LEN(TRIM(G235))=0,0,LEN(TRIM(G235))-LEN(SUBSTITUTE(TRIM(G235)," ",""))+1)</f>
-      </c>
-      <c r="J235" s="3">
-        <f>IF(LEN(TRIM(H235))=0,0,LEN(TRIM(H235))-LEN(SUBSTITUTE(TRIM(H235)," ",""))+1)</f>
-      </c>
-      <c r="K235" s="3">
-        <f>LEN(G235)</f>
-      </c>
-      <c r="L235" s="3">
-        <f>LEN(H235)</f>
-      </c>
-      <c r="M235" s="3">
-        <f>IF(COUNTIF($G:$G,G235)&gt;1,"DUP","")</f>
-      </c>
-      <c r="N235" s="3">
-        <f>IF(COUNTIF($H:$H,H235)&gt;1,"DUP","")</f>
-      </c>
-      <c r="O235" s="3">
-        <f>IF(LEFT(B235,LEN(C235))=C235,"OK","CHECK")</f>
-      </c>
-      <c r="P235" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Review</t>
-        </is>
-      </c>
-      <c r="Q235" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="R235" s="5">
-        <f>IF(OR(M235="DUP",N235="DUP",O235="CHECK"),"CHECK","")</f>
-      </c>
-      <c r="S235" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="T235" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="U235" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="236">
-      <c r="A236" s="2">
-        <v>170</v>
-      </c>
-      <c r="B236" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.below_push.minimal.1</t>
-        </is>
-      </c>
-      <c r="C236" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.below_push</t>
-        </is>
-      </c>
-      <c r="D236" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.below_push.minimal</t>
-        </is>
-      </c>
-      <c r="E236" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">personal_trainer</t>
-        </is>
-      </c>
-      <c r="F236" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">core</t>
-        </is>
-      </c>
-      <c r="G236" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">You're moving. Add a little.</t>
-        </is>
-      </c>
-      <c r="H236" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du er i gang. Litt opp.</t>
-        </is>
-      </c>
-      <c r="I236" s="3">
-        <f>IF(LEN(TRIM(G236))=0,0,LEN(TRIM(G236))-LEN(SUBSTITUTE(TRIM(G236)," ",""))+1)</f>
-      </c>
-      <c r="J236" s="3">
-        <f>IF(LEN(TRIM(H236))=0,0,LEN(TRIM(H236))-LEN(SUBSTITUTE(TRIM(H236)," ",""))+1)</f>
-      </c>
-      <c r="K236" s="3">
-        <f>LEN(G236)</f>
-      </c>
-      <c r="L236" s="3">
-        <f>LEN(H236)</f>
-      </c>
-      <c r="M236" s="3">
-        <f>IF(COUNTIF($G:$G,G236)&gt;1,"DUP","")</f>
-      </c>
-      <c r="N236" s="3">
-        <f>IF(COUNTIF($H:$H,H236)&gt;1,"DUP","")</f>
-      </c>
-      <c r="O236" s="3">
-        <f>IF(LEFT(B236,LEN(C236))=C236,"OK","CHECK")</f>
-      </c>
-      <c r="P236" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Review</t>
-        </is>
-      </c>
-      <c r="Q236" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="R236" s="5">
-        <f>IF(OR(M236="DUP",N236="DUP",O236="CHECK"),"CHECK","")</f>
-      </c>
-      <c r="S236" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="T236" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="U236" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="237">
-      <c r="A237" s="2">
-        <v>200</v>
-      </c>
-      <c r="B237" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.breath.easy_run.1</t>
-        </is>
-      </c>
-      <c r="C237" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.breath</t>
-        </is>
-      </c>
-      <c r="D237" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.breath.easy_run</t>
-        </is>
-      </c>
-      <c r="E237" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">personal_trainer</t>
-        </is>
-      </c>
-      <c r="F237" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">core</t>
-        </is>
-      </c>
-      <c r="G237" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Match your breathing to your pace.</t>
-        </is>
-      </c>
-      <c r="H237" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tilpass pusten til tempoet.</t>
-        </is>
-      </c>
-      <c r="I237" s="3">
-        <f>IF(LEN(TRIM(G237))=0,0,LEN(TRIM(G237))-LEN(SUBSTITUTE(TRIM(G237)," ",""))+1)</f>
-      </c>
-      <c r="J237" s="3">
-        <f>IF(LEN(TRIM(H237))=0,0,LEN(TRIM(H237))-LEN(SUBSTITUTE(TRIM(H237)," ",""))+1)</f>
-      </c>
-      <c r="K237" s="3">
-        <f>LEN(G237)</f>
-      </c>
-      <c r="L237" s="3">
-        <f>LEN(H237)</f>
-      </c>
-      <c r="M237" s="3">
-        <f>IF(COUNTIF($G:$G,G237)&gt;1,"DUP","")</f>
-      </c>
-      <c r="N237" s="3">
-        <f>IF(COUNTIF($H:$H,H237)&gt;1,"DUP","")</f>
-      </c>
-      <c r="O237" s="3">
-        <f>IF(LEFT(B237,LEN(C237))=C237,"OK","CHECK")</f>
-      </c>
-      <c r="P237" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Review</t>
-        </is>
-      </c>
-      <c r="Q237" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="R237" s="5">
-        <f>IF(OR(M237="DUP",N237="DUP",O237="CHECK"),"CHECK","")</f>
-      </c>
-      <c r="S237" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="T237" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="U237" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="238">
-      <c r="A238" s="2">
-        <v>201</v>
-      </c>
-      <c r="B238" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.breath.easy_run.2</t>
-        </is>
-      </c>
-      <c r="C238" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.breath</t>
-        </is>
-      </c>
-      <c r="D238" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.breath.easy_run</t>
-        </is>
-      </c>
-      <c r="E238" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">personal_trainer</t>
-        </is>
-      </c>
-      <c r="F238" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">core</t>
-        </is>
-      </c>
-      <c r="G238" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Smooth breaths. You're doing well.</t>
-        </is>
-      </c>
-      <c r="H238" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jevn pust. Du gjør det bra.</t>
-        </is>
-      </c>
-      <c r="I238" s="3">
-        <f>IF(LEN(TRIM(G238))=0,0,LEN(TRIM(G238))-LEN(SUBSTITUTE(TRIM(G238)," ",""))+1)</f>
-      </c>
-      <c r="J238" s="3">
-        <f>IF(LEN(TRIM(H238))=0,0,LEN(TRIM(H238))-LEN(SUBSTITUTE(TRIM(H238)," ",""))+1)</f>
-      </c>
-      <c r="K238" s="3">
-        <f>LEN(G238)</f>
-      </c>
-      <c r="L238" s="3">
-        <f>LEN(H238)</f>
-      </c>
-      <c r="M238" s="3">
-        <f>IF(COUNTIF($G:$G,G238)&gt;1,"DUP","")</f>
-      </c>
-      <c r="N238" s="3">
-        <f>IF(COUNTIF($H:$H,H238)&gt;1,"DUP","")</f>
-      </c>
-      <c r="O238" s="3">
-        <f>IF(LEFT(B238,LEN(C238))=C238,"OK","CHECK")</f>
-      </c>
-      <c r="P238" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Review</t>
-        </is>
-      </c>
-      <c r="Q238" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="R238" s="5">
-        <f>IF(OR(M238="DUP",N238="DUP",O238="CHECK"),"CHECK","")</f>
-      </c>
-      <c r="S238" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="T238" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="U238" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="239">
-      <c r="A239" s="2">
-        <v>203</v>
-      </c>
-      <c r="B239" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.breath.recovery.1</t>
-        </is>
-      </c>
-      <c r="C239" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.breath</t>
-        </is>
-      </c>
-      <c r="D239" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.breath.recovery</t>
-        </is>
-      </c>
-      <c r="E239" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">personal_trainer</t>
-        </is>
-      </c>
-      <c r="F239" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">core</t>
-        </is>
-      </c>
-      <c r="G239" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Slow your breathing down.</t>
-        </is>
-      </c>
-      <c r="H239" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Senk pustetakten.</t>
-        </is>
-      </c>
-      <c r="I239" s="3">
-        <f>IF(LEN(TRIM(G239))=0,0,LEN(TRIM(G239))-LEN(SUBSTITUTE(TRIM(G239)," ",""))+1)</f>
-      </c>
-      <c r="J239" s="3">
-        <f>IF(LEN(TRIM(H239))=0,0,LEN(TRIM(H239))-LEN(SUBSTITUTE(TRIM(H239)," ",""))+1)</f>
-      </c>
-      <c r="K239" s="3">
-        <f>LEN(G239)</f>
-      </c>
-      <c r="L239" s="3">
-        <f>LEN(H239)</f>
-      </c>
-      <c r="M239" s="3">
-        <f>IF(COUNTIF($G:$G,G239)&gt;1,"DUP","")</f>
-      </c>
-      <c r="N239" s="3">
-        <f>IF(COUNTIF($H:$H,H239)&gt;1,"DUP","")</f>
-      </c>
-      <c r="O239" s="3">
-        <f>IF(LEFT(B239,LEN(C239))=C239,"OK","CHECK")</f>
-      </c>
-      <c r="P239" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Review</t>
-        </is>
-      </c>
-      <c r="Q239" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="R239" s="5">
-        <f>IF(OR(M239="DUP",N239="DUP",O239="CHECK"),"CHECK","")</f>
-      </c>
-      <c r="S239" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="T239" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="U239" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="240">
-      <c r="A240" s="2">
-        <v>202</v>
-      </c>
-      <c r="B240" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.breath.work.1</t>
-        </is>
-      </c>
-      <c r="C240" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.breath</t>
-        </is>
-      </c>
-      <c r="D240" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.breath.work</t>
-        </is>
-      </c>
-      <c r="E240" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">personal_trainer</t>
-        </is>
-      </c>
-      <c r="F240" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">core</t>
-        </is>
-      </c>
-      <c r="G240" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Breathe through the effort.</t>
-        </is>
-      </c>
-      <c r="H240" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Herlig</t>
-        </is>
-      </c>
-      <c r="I240" s="3">
-        <f>IF(LEN(TRIM(G240))=0,0,LEN(TRIM(G240))-LEN(SUBSTITUTE(TRIM(G240)," ",""))+1)</f>
-      </c>
-      <c r="J240" s="3">
-        <f>IF(LEN(TRIM(H240))=0,0,LEN(TRIM(H240))-LEN(SUBSTITUTE(TRIM(H240)," ",""))+1)</f>
-      </c>
-      <c r="K240" s="3">
-        <f>LEN(G240)</f>
-      </c>
-      <c r="L240" s="3">
-        <f>LEN(H240)</f>
-      </c>
-      <c r="M240" s="3">
-        <f>IF(COUNTIF($G:$G,G240)&gt;1,"DUP","")</f>
-      </c>
-      <c r="N240" s="3">
-        <f>IF(COUNTIF($H:$H,H240)&gt;1,"DUP","")</f>
-      </c>
-      <c r="O240" s="3">
-        <f>IF(LEFT(B240,LEN(C240))=C240,"OK","CHECK")</f>
-      </c>
-      <c r="P240" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Review</t>
-        </is>
-      </c>
-      <c r="Q240" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="R240" s="5">
-        <f>IF(OR(M240="DUP",N240="DUP",O240="CHECK"),"CHECK","")</f>
-      </c>
-      <c r="S240" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="T240" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="U240" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="241">
-      <c r="A241" s="2">
-        <v>193</v>
-      </c>
-      <c r="B241" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel.easy_run.1</t>
-        </is>
-      </c>
-      <c r="C241" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel</t>
-        </is>
-      </c>
-      <c r="D241" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel.easy_run</t>
-        </is>
-      </c>
-      <c r="E241" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">personal_trainer</t>
-        </is>
-      </c>
-      <c r="F241" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">core</t>
-        </is>
-      </c>
-      <c r="G241" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Steady effort. Stay comfortable.</t>
-        </is>
-      </c>
-      <c r="H241" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jevn innsats. Hold det behagelig.</t>
-        </is>
-      </c>
-      <c r="I241" s="3">
-        <f>IF(LEN(TRIM(G241))=0,0,LEN(TRIM(G241))-LEN(SUBSTITUTE(TRIM(G241)," ",""))+1)</f>
-      </c>
-      <c r="J241" s="3">
-        <f>IF(LEN(TRIM(H241))=0,0,LEN(TRIM(H241))-LEN(SUBSTITUTE(TRIM(H241)," ",""))+1)</f>
-      </c>
-      <c r="K241" s="3">
-        <f>LEN(G241)</f>
-      </c>
-      <c r="L241" s="3">
-        <f>LEN(H241)</f>
-      </c>
-      <c r="M241" s="3">
-        <f>IF(COUNTIF($G:$G,G241)&gt;1,"DUP","")</f>
-      </c>
-      <c r="N241" s="3">
-        <f>IF(COUNTIF($H:$H,H241)&gt;1,"DUP","")</f>
-      </c>
-      <c r="O241" s="3">
-        <f>IF(LEFT(B241,LEN(C241))=C241,"OK","CHECK")</f>
-      </c>
-      <c r="P241" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Review</t>
-        </is>
-      </c>
-      <c r="Q241" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="R241" s="5">
-        <f>IF(OR(M241="DUP",N241="DUP",O241="CHECK"),"CHECK","")</f>
-      </c>
-      <c r="S241" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="T241" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="U241" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="242">
-      <c r="A242" s="2">
-        <v>194</v>
-      </c>
-      <c r="B242" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel.easy_run.2</t>
-        </is>
-      </c>
-      <c r="C242" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel</t>
-        </is>
-      </c>
-      <c r="D242" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel.easy_run</t>
-        </is>
-      </c>
-      <c r="E242" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">personal_trainer</t>
-        </is>
-      </c>
-      <c r="F242" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">core</t>
-        </is>
-      </c>
-      <c r="G242" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Find your rhythm and hold it.</t>
-        </is>
-      </c>
-      <c r="H242" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Finn rytmen din og hold den.</t>
-        </is>
-      </c>
-      <c r="I242" s="3">
-        <f>IF(LEN(TRIM(G242))=0,0,LEN(TRIM(G242))-LEN(SUBSTITUTE(TRIM(G242)," ",""))+1)</f>
-      </c>
-      <c r="J242" s="3">
-        <f>IF(LEN(TRIM(H242))=0,0,LEN(TRIM(H242))-LEN(SUBSTITUTE(TRIM(H242)," ",""))+1)</f>
-      </c>
-      <c r="K242" s="3">
-        <f>LEN(G242)</f>
-      </c>
-      <c r="L242" s="3">
-        <f>LEN(H242)</f>
-      </c>
-      <c r="M242" s="3">
-        <f>IF(COUNTIF($G:$G,G242)&gt;1,"DUP","")</f>
-      </c>
-      <c r="N242" s="3">
-        <f>IF(COUNTIF($H:$H,H242)&gt;1,"DUP","")</f>
-      </c>
-      <c r="O242" s="3">
-        <f>IF(LEFT(B242,LEN(C242))=C242,"OK","CHECK")</f>
-      </c>
-      <c r="P242" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Review</t>
-        </is>
-      </c>
-      <c r="Q242" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="R242" s="5">
-        <f>IF(OR(M242="DUP",N242="DUP",O242="CHECK"),"CHECK","")</f>
-      </c>
-      <c r="S242" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="T242" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="U242" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" s="2">
-        <v>195</v>
-      </c>
-      <c r="B243" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel.easy_run.3</t>
-        </is>
-      </c>
-      <c r="C243" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel</t>
-        </is>
-      </c>
-      <c r="D243" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel.easy_run</t>
-        </is>
-      </c>
-      <c r="E243" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">personal_trainer</t>
-        </is>
-      </c>
-      <c r="F243" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">core</t>
-        </is>
-      </c>
-      <c r="G243" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Easy and controlled. You set the pace.</t>
-        </is>
-      </c>
-      <c r="H243" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rolig og kontrollert. Du bestemmer tempoet.</t>
-        </is>
-      </c>
-      <c r="I243" s="3">
-        <f>IF(LEN(TRIM(G243))=0,0,LEN(TRIM(G243))-LEN(SUBSTITUTE(TRIM(G243)," ",""))+1)</f>
-      </c>
-      <c r="J243" s="3">
-        <f>IF(LEN(TRIM(H243))=0,0,LEN(TRIM(H243))-LEN(SUBSTITUTE(TRIM(H243)," ",""))+1)</f>
-      </c>
-      <c r="K243" s="3">
-        <f>LEN(G243)</f>
-      </c>
-      <c r="L243" s="3">
-        <f>LEN(H243)</f>
-      </c>
-      <c r="M243" s="3">
-        <f>IF(COUNTIF($G:$G,G243)&gt;1,"DUP","")</f>
-      </c>
-      <c r="N243" s="3">
-        <f>IF(COUNTIF($H:$H,H243)&gt;1,"DUP","")</f>
-      </c>
-      <c r="O243" s="3">
-        <f>IF(LEFT(B243,LEN(C243))=C243,"OK","CHECK")</f>
-      </c>
-      <c r="P243" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Review</t>
-        </is>
-      </c>
-      <c r="Q243" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="R243" s="5">
-        <f>IF(OR(M243="DUP",N243="DUP",O243="CHECK"),"CHECK","")</f>
-      </c>
-      <c r="S243" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="T243" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="U243" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="244">
-      <c r="A244" s="2">
-        <v>198</v>
-      </c>
-      <c r="B244" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel.recovery.1</t>
-        </is>
-      </c>
-      <c r="C244" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel</t>
-        </is>
-      </c>
-      <c r="D244" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel.recovery</t>
-        </is>
-      </c>
-      <c r="E244" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">personal_trainer</t>
-        </is>
-      </c>
-      <c r="F244" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">core</t>
-        </is>
-      </c>
-      <c r="G244" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ease off. Let your body recover.</t>
-        </is>
-      </c>
-      <c r="H244" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Slipp av. La kroppen hente seg inn.</t>
-        </is>
-      </c>
-      <c r="I244" s="3">
-        <f>IF(LEN(TRIM(G244))=0,0,LEN(TRIM(G244))-LEN(SUBSTITUTE(TRIM(G244)," ",""))+1)</f>
-      </c>
-      <c r="J244" s="3">
-        <f>IF(LEN(TRIM(H244))=0,0,LEN(TRIM(H244))-LEN(SUBSTITUTE(TRIM(H244)," ",""))+1)</f>
-      </c>
-      <c r="K244" s="3">
-        <f>LEN(G244)</f>
-      </c>
-      <c r="L244" s="3">
-        <f>LEN(H244)</f>
-      </c>
-      <c r="M244" s="3">
-        <f>IF(COUNTIF($G:$G,G244)&gt;1,"DUP","")</f>
-      </c>
-      <c r="N244" s="3">
-        <f>IF(COUNTIF($H:$H,H244)&gt;1,"DUP","")</f>
-      </c>
-      <c r="O244" s="3">
-        <f>IF(LEFT(B244,LEN(C244))=C244,"OK","CHECK")</f>
-      </c>
-      <c r="P244" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Review</t>
-        </is>
-      </c>
-      <c r="Q244" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="R244" s="5">
-        <f>IF(OR(M244="DUP",N244="DUP",O244="CHECK"),"CHECK","")</f>
-      </c>
-      <c r="S244" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="T244" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="U244" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="245">
-      <c r="A245" s="2">
-        <v>199</v>
-      </c>
-      <c r="B245" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel.recovery.2</t>
-        </is>
-      </c>
-      <c r="C245" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel</t>
-        </is>
-      </c>
-      <c r="D245" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel.recovery</t>
-        </is>
-      </c>
-      <c r="E245" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">personal_trainer</t>
-        </is>
-      </c>
-      <c r="F245" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">core</t>
-        </is>
-      </c>
-      <c r="G245" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Relax and breathe. Recovery counts.</t>
-        </is>
-      </c>
-      <c r="H245" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Slapp av og pust. Hvile teller.</t>
-        </is>
-      </c>
-      <c r="I245" s="3">
-        <f>IF(LEN(TRIM(G245))=0,0,LEN(TRIM(G245))-LEN(SUBSTITUTE(TRIM(G245)," ",""))+1)</f>
-      </c>
-      <c r="J245" s="3">
-        <f>IF(LEN(TRIM(H245))=0,0,LEN(TRIM(H245))-LEN(SUBSTITUTE(TRIM(H245)," ",""))+1)</f>
-      </c>
-      <c r="K245" s="3">
-        <f>LEN(G245)</f>
-      </c>
-      <c r="L245" s="3">
-        <f>LEN(H245)</f>
-      </c>
-      <c r="M245" s="3">
-        <f>IF(COUNTIF($G:$G,G245)&gt;1,"DUP","")</f>
-      </c>
-      <c r="N245" s="3">
-        <f>IF(COUNTIF($H:$H,H245)&gt;1,"DUP","")</f>
-      </c>
-      <c r="O245" s="3">
-        <f>IF(LEFT(B245,LEN(C245))=C245,"OK","CHECK")</f>
-      </c>
-      <c r="P245" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Review</t>
-        </is>
-      </c>
-      <c r="Q245" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="R245" s="5">
-        <f>IF(OR(M245="DUP",N245="DUP",O245="CHECK"),"CHECK","")</f>
-      </c>
-      <c r="S245" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="T245" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="U245" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" s="2">
-        <v>196</v>
-      </c>
-      <c r="B246" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel.work.1</t>
-        </is>
-      </c>
-      <c r="C246" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel</t>
-        </is>
-      </c>
-      <c r="D246" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel.work</t>
-        </is>
-      </c>
-      <c r="E246" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">personal_trainer</t>
-        </is>
-      </c>
-      <c r="F246" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">core</t>
-        </is>
-      </c>
-      <c r="G246" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Push hard but controlled.</t>
-        </is>
-      </c>
-      <c r="H246" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hold en jevn rytme</t>
-        </is>
-      </c>
-      <c r="I246" s="3">
-        <f>IF(LEN(TRIM(G246))=0,0,LEN(TRIM(G246))-LEN(SUBSTITUTE(TRIM(G246)," ",""))+1)</f>
-      </c>
-      <c r="J246" s="3">
-        <f>IF(LEN(TRIM(H246))=0,0,LEN(TRIM(H246))-LEN(SUBSTITUTE(TRIM(H246)," ",""))+1)</f>
-      </c>
-      <c r="K246" s="3">
-        <f>LEN(G246)</f>
-      </c>
-      <c r="L246" s="3">
-        <f>LEN(H246)</f>
-      </c>
-      <c r="M246" s="3">
-        <f>IF(COUNTIF($G:$G,G246)&gt;1,"DUP","")</f>
-      </c>
-      <c r="N246" s="3">
-        <f>IF(COUNTIF($H:$H,H246)&gt;1,"DUP","")</f>
-      </c>
-      <c r="O246" s="3">
-        <f>IF(LEFT(B246,LEN(C246))=C246,"OK","CHECK")</f>
-      </c>
-      <c r="P246" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Review</t>
-        </is>
-      </c>
-      <c r="Q246" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="R246" s="5">
-        <f>IF(OR(M246="DUP",N246="DUP",O246="CHECK"),"CHECK","")</f>
-      </c>
-      <c r="S246" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="T246" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="U246" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="247">
-      <c r="A247" s="2">
-        <v>197</v>
-      </c>
-      <c r="B247" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel.work.2</t>
-        </is>
-      </c>
-      <c r="C247" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel</t>
-        </is>
-      </c>
-      <c r="D247" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">zone.feel.work</t>
-        </is>
-      </c>
-      <c r="E247" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">personal_trainer</t>
-        </is>
-      </c>
-      <c r="F247" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">core</t>
-        </is>
-      </c>
-      <c r="G247" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Strong effort now. Stay focused.</t>
-        </is>
-      </c>
-      <c r="H247" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sterk innsats nå. Hold fokus.</t>
-        </is>
-      </c>
-      <c r="I247" s="3">
-        <f>IF(LEN(TRIM(G247))=0,0,LEN(TRIM(G247))-LEN(SUBSTITUTE(TRIM(G247)," ",""))+1)</f>
-      </c>
-      <c r="J247" s="3">
-        <f>IF(LEN(TRIM(H247))=0,0,LEN(TRIM(H247))-LEN(SUBSTITUTE(TRIM(H247)," ",""))+1)</f>
-      </c>
-      <c r="K247" s="3">
-        <f>LEN(G247)</f>
-      </c>
-      <c r="L247" s="3">
-        <f>LEN(H247)</f>
-      </c>
-      <c r="M247" s="3">
-        <f>IF(COUNTIF($G:$G,G247)&gt;1,"DUP","")</f>
-      </c>
-      <c r="N247" s="3">
-        <f>IF(COUNTIF($H:$H,H247)&gt;1,"DUP","")</f>
-      </c>
-      <c r="O247" s="3">
-        <f>IF(LEFT(B247,LEN(C247))=C247,"OK","CHECK")</f>
-      </c>
-      <c r="P247" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Review</t>
-        </is>
-      </c>
-      <c r="Q247" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="R247" s="5">
-        <f>IF(OR(M247="DUP",N247="DUP",O247="CHECK"),"CHECK","")</f>
-      </c>
-      <c r="S247" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="T247" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="U247" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:U247"/>
+  <autoFilter ref="A1:U231"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="P2:P247">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="P2:P231">
       <formula1>"Review,Keep,Edit,Remove,Needs Translation"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>